<commit_message>
Added Completed this session (March 27, 2026) with a full explanation of the RM 1.5 site name matching fix Task list renumbered: CDX re-upload is now the sole immediate priority (blocking issue resolved), followed by script extraction, historical corrections, and inline tables Known Data Issues: marked the 11 missing monitoring_location_id rows as resolved, and updated the output CSV note to reflect the clean March 27 re-render Removed the stale CMB eval = F note and replaced with the actual result (52.2% project-wide)
</commit_message>
<xml_diff>
--- a/other/input/wqx_templates/sgs_site_names_matching_table_manual_edit.xlsx
+++ b/other/input/wqx_templates/sgs_site_names_matching_table_manual_edit.xlsx
@@ -1,31 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd0dd052dcf49e10/Documents/GitHub_Local/kenai-river-wqx/other/input/AQWMS/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_EE66614BA1A2EAAC1296813F4239D4396297A70B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A95064CD-EE3F-41E4-9412-C19CB2BD83C7}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="13860" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>Monitoring Location Name</t>
   </si>
@@ -343,13 +331,23 @@
   </si>
   <si>
     <t>RM_21_Soldotna_Bridge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kenai River - River Mile 1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KR RM 1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RM1.5_Kenai_City_Dock</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -358,12 +356,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -668,16 +666,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="44.140625" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="33.42578125" customWidth="1"/>
+    <col min="1" max="1" width="44.140625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -688,7 +686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -699,7 +697,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -710,7 +708,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -721,7 +719,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -732,7 +730,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -743,7 +741,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -754,7 +752,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -765,7 +763,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -776,7 +774,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -787,7 +785,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -801,7 +799,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -812,7 +810,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -823,7 +821,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -834,7 +832,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -845,7 +843,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -859,7 +857,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -870,7 +868,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -881,7 +879,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -892,7 +890,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -903,7 +901,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -914,7 +912,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -925,7 +923,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -936,7 +934,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="A24" t="s">
         <v>9</v>
       </c>
@@ -947,7 +945,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="A25" t="s">
         <v>9</v>
       </c>
@@ -958,7 +956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="A26" t="s">
         <v>10</v>
       </c>
@@ -969,7 +967,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -983,7 +981,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28">
       <c r="A28" t="s">
         <v>10</v>
       </c>
@@ -997,7 +995,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -1008,7 +1006,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -1019,7 +1017,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -1030,7 +1028,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -1044,7 +1042,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -1055,7 +1053,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -1066,7 +1064,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -1077,7 +1075,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -1088,7 +1086,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37">
       <c r="A37" t="s">
         <v>15</v>
       </c>
@@ -1099,7 +1097,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -1110,7 +1108,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39">
       <c r="A39" t="s">
         <v>15</v>
       </c>
@@ -1124,7 +1122,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40">
       <c r="A40" t="s">
         <v>16</v>
       </c>
@@ -1135,7 +1133,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -1149,7 +1147,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -1163,7 +1161,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43">
       <c r="A43" t="s">
         <v>17</v>
       </c>
@@ -1180,7 +1178,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44">
       <c r="A44" t="s">
         <v>17</v>
       </c>
@@ -1191,7 +1189,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -1202,7 +1200,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -1213,7 +1211,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -1224,7 +1222,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48">
       <c r="A48" t="s">
         <v>18</v>
       </c>
@@ -1235,7 +1233,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49">
       <c r="A49" t="s">
         <v>18</v>
       </c>
@@ -1246,7 +1244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50">
       <c r="A50" t="s">
         <v>23</v>
       </c>
@@ -1260,7 +1258,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51">
       <c r="A51" t="s">
         <v>23</v>
       </c>
@@ -1271,7 +1269,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -1285,7 +1283,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53">
       <c r="A53" t="s">
         <v>19</v>
       </c>
@@ -1296,7 +1294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54">
       <c r="A54" t="s">
         <v>20</v>
       </c>
@@ -1307,7 +1305,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55">
       <c r="A55" t="s">
         <v>20</v>
       </c>
@@ -1318,7 +1316,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56">
       <c r="A56" t="s">
         <v>2</v>
       </c>
@@ -1329,7 +1327,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -1340,7 +1338,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -1351,7 +1349,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59">
       <c r="A59" t="s">
         <v>15</v>
       </c>
@@ -1362,11 +1360,19 @@
         <v>78</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>106</v>
+      </c>
+      <c r="B60" t="s">
+        <v>107</v>
+      </c>
+      <c r="C60" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
-    <sortCondition ref="B2:B73"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>